<commit_message>
implemented processing data from JSON Instructions
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\DEV\Rapport-Generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DF9BA4-EE1C-4166-BC41-6F48CB40AAF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08478C2-9F00-4CAB-9990-8C03D690F9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>date</t>
   </si>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>Requires follow-up visit</t>
-  </si>
-  <si>
-    <t>Spiceis</t>
   </si>
 </sst>
 </file>
@@ -475,9 +472,7 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3">

</xml_diff>